<commit_message>
Ignored errrors in sorted data
</commit_message>
<xml_diff>
--- a/Experiment/Results/FramerateSorted.xlsx
+++ b/Experiment/Results/FramerateSorted.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Howest\GD_J3_S2\Gradwork_2.0\Gradwork\Experiment\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F2CBC9B-78A7-4E8A-B0B9-B4153E1D7FAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A712D1-3E82-42AF-9D45-BA37ED3DA92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-10790" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SSAO" sheetId="1" r:id="rId1"/>
@@ -1561,6 +1561,9 @@
     <sortCondition ref="E4:X4"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="D4:D15" formulaRange="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -1882,7 +1885,7 @@
       <c r="C7" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="3">
         <f t="shared" si="0"/>
         <v>0.25077760000000004</v>
       </c>
@@ -1954,7 +1957,7 @@
       <c r="C8" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="3">
         <f t="shared" si="0"/>
         <v>0.91135999999999995</v>
       </c>
@@ -2026,7 +2029,7 @@
       <c r="C9" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="3">
         <f t="shared" si="0"/>
         <v>3.3596415999999998</v>
       </c>
@@ -2314,7 +2317,7 @@
       <c r="C13" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="3">
         <f t="shared" si="0"/>
         <v>11.729510400000001</v>
       </c>
@@ -2386,7 +2389,7 @@
       <c r="C14" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="3">
         <f t="shared" si="0"/>
         <v>39.007024799999996</v>
       </c>
@@ -2458,7 +2461,7 @@
       <c r="C15" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="3">
         <f t="shared" si="0"/>
         <v>178.87744000000001</v>
       </c>
@@ -2528,6 +2531,9 @@
     <sortCondition ref="E3:X3"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="D4:D15" formulaRange="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -2537,6 +2543,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="11" width="11" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
@@ -3490,5 +3497,8 @@
     <sortCondition ref="E15:X15"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="D4 D5:D15" formulaRange="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>